<commit_message>
fix(changeover): snapshot-first, state mapping BATTERY/INPUT/SAFE, MillisecondsToTicks, remove duplicate Excel - snapshot NULL/invalid first: preserve state/PB11, reset timers, fault does not trigger FAULT when invalid, invalid time not counted - fault only when snapshot valid -> FAULT no pin - state: valid+input false->BATTERY, valid+input true->INPUT, after cut->SAFE, after reconnect->INPUT, no IDLE for valid - 3000ms via func__Rtos_MillisecondsToTicks, no tick=1ms assumption - keep only Changeover_Board_Validation.xlsx, remove Changeover_Validation.xlsx, add fault+invalid scenario CO-021
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -682,10 +682,10 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T24"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -904,7 +904,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>BOOT/IDLE حفظ</t>
+          <t>BOOT حفظ (تغییر نکند)</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>IDLE/BATTERY</t>
+          <t>BATTERY</t>
         </is>
       </c>
       <c r="L7" s="8" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>IDLE</t>
+          <t>INPUT</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>IDLE</t>
+          <t>INPUT</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -2406,6 +2406,84 @@
       <c r="R24" s="9" t="inlineStr"/>
       <c r="S24" s="9" t="inlineStr"/>
       <c r="T24" s="9" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>CO-021</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Fault با snapshot نامعتبر</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>fault≠0 با snapshot.valid=false (v=20700), بررسی اولویت invalid</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>20700</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>FAULT_ADC</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>PB11 حفظ</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>BOOT حفظ</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>در invalid، fault نباید FAULT شود</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr"/>
+      <c r="N25" s="10" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="O25" s="9" t="inlineStr"/>
+      <c r="P25" s="9" t="inlineStr"/>
+      <c r="Q25" s="9" t="inlineStr"/>
+      <c r="R25" s="9" t="inlineStr"/>
+      <c r="S25" s="9" t="inlineStr"/>
+      <c r="T25" s="9" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>

</xml_diff>

<commit_message>
fix(validation): correct Excel content per c8c0265 base
- Measurement MS-004: remove Wait/?, define I channels 610 for 486mA, V channels 2482
- Measurement MS-020: remove Actually/?, set V24 36882 V12 19897 Current 3267
- Measurement MS-021: remove Wait/?, set pin 2147mV counts 2665 V24 24000
- Changeover CO-013: remove Actually/?, set before 3000 SAFE PB11 Low after INPUT PB11 High
- Buzzer BZ-010: remove ?/Actually, set dutyWindow1200 ON1200 tail58800 nextCheck120
- Remove all Wait/Actually/?/maybe/TBD from workbooks
- Final page commit set to c8c0265 (real build) not hard-coded c6b084f
- Confirm MODULE_CHANGEOVER=1 per c8c0265 (cherry-picked)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -1016,7 +1016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1922,12 +1922,12 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>پس از 2500ms هنوز SAFE High? Actually PB11 Low؛ پس از 3000ms PB11 High (وصل) و state=INPUT. PASS: reconnect پس از 3000ms. FAIL: reconnect زود یا عدم reconnect.</t>
+          <t>قبل از 3000ms: SAFE و PB11 Low؛ بعد از 3000ms: INPUT و PB11 High. PASS: reconnect پس از 3000ms با PB11 High. FAIL: reconnect زود یا PB11 Low ماندن.</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>PASS: 3000ms → INPUT High. FAIL: early or no reconnect.</t>
+          <t>PASS: قبل 3000 SAFE Low، بعد 3000 INPUT High. FAIL: early or no reconnect.</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr"/>
@@ -2504,10 +2504,6 @@
       <c r="O26" s="20" t="inlineStr"/>
       <c r="P26" s="20" t="inlineStr"/>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <autoFilter ref="A4:P26"/>
   <mergeCells count="3">
@@ -3339,7 +3335,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>c6b084f28f2c507cfd342e5dbd0dbd8e45686772</t>
+          <t>c8c0265e2c3086702f1369b50b467011fd967a94</t>
         </is>
       </c>
       <c r="C6" s="26" t="inlineStr">

</xml_diff>

<commit_message>
state machines: one coloured workbook per module linked from each module validation file, drop the duplicated scenario 1-3 flow lines in the panel
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel help text: drop the duplicated flow line from every scenario card, reflow the help blocks one definition per line, close number-unit gaps for RTL
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel help text: finish the sweep - every run-on help block now reads one definition per line with its reason split out
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: close the scenario-3 ladder section header (its help text and inputs were rendering inside a bold header), add a markup invariant
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: centre the charge-scenario table, close every number-unit gap in Persian text (markup, JS output and docs), guard it in the audit
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: centre the bench scenario table too, restore the space where a digit is a channel index or the text is English, refine the unit-gap invariant
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: move every unit inside its isolated number span so number+unit is one unbreakable LTR run
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: Persian unit words inside prose (no more bidi flips), every table centred, box labels left as they were
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: the sweep row captions sit beside their boxes instead of above them
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
panel: scenario 1 beep summary prints the gap value instead of the word, sweep captions pinned beside their boxes
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -13,6 +13,7 @@
     <sheet name="ثبت ایراد" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تأیید نهایی" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فهرست‌ها" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="ماشین حالت" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه تست'!$A$4:$P$26</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,29 @@
     <font>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -160,8 +182,13 @@
         <bgColor rgb="00E9EDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -227,11 +254,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009DB7E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="009DB7E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="009DB7E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009DB7E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +355,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3950,4 +4003,85 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>ماشین حالت ماژول تغییر مسیر (Changeover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>حالت‌ها و گذارهای همین ماژول</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Changeover_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ماشین حالت کل برنامه (نمای سیستمی)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>../../../Documentation/System_State_Machine.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>راهنمای رنگ‌ها</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>بازتولید</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>python3 tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Review Changeover: validation sheet refers to the internal latch, not the removed UI flag
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -778,7 +778,7 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>این فایل برای اعتبارسنجی منطق Changeover تهیه شده است: بررسی snapshot.valid، fault_mask، input_present، v_bat24_mv، فلگ UI و تایمر 3000ms.</t>
+          <t>این فایل برای اعتبارسنجی منطق Changeover تهیه شده است: بررسی snapshot.valid، fault_mask، input_present، v_bat24_mv، قفل داخلی باتری کم و تایمر 3000ms.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>۳) snapshot را تزریق کن: valid، v_bat24_mv، input_present و فلگ UI را ست کن؛ fault_mask را از Fault اعمال کن.</t>
+          <t>۳) snapshot را تزریق کن: valid، v_bat24_mv، input_present و قفل داخلی باتری کم را ست کن؛ fault_mask را از Fault اعمال کن.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: thermal rest 1h->10min + 30s input stable reconnect + Vin 22-30V range
- Charger: add CHG_INPUT_VALID_MAX_MV 30000, input check min+max (was only min)
- Charger: add THERMAL_REST state, per-channel timers 1h continuous at max current (bulkMax-50mA) -> 10min rest PWM=0 relay closed, preserve in SafeIdle
- Changeover: add CHANGEOVER_INPUT_STABLE_MS 30000, require input stable 30s extra before reconnect (user order 2026-10-12), plus existing 3s voltage filter = 33s total
- Host test Changeover: update to expect 30s+3s
- README updates for both modules
- Validation excels: CO-024 30s test, CH-036 thermal, CH-037 Vin range, CH-038 SafeIdle preserve
- audit 449 PASS, ai_rules ALL PASS, host tests PASS

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -1091,7 +1091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2635,17 +2635,73 @@
           <t>نیاز به تکرار</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>62f3782</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
           <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CO-024</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>وصل مجدد 30s پایداری ورودی</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>برد در SAFE پس از قطع، v_bat=24V</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ورودی را وصل و 30s نگه دار سپس 3s ولتاژ 21200</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>input=true v=24000</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>33s</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>بعد 30s پایداری + 3s ولتاژ، PB11 High-&gt;Low و INPUT</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>PASS: PB11 بعد 33s وصل، قبلش SAFE. FAIL: وصل زودتر از 30s</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>نیاز به تکرار</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>thermal+30s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(validation): sweep all 30 workbooks - last wrong-row date formulas fixed
Follow-up full sweep (user asked whether EVERY file was checked):
scanned all 30 xlsx, every sheet, all 727 formulas. Found 12 more
date formulas keyed to the wrong row that the practical-sheet
rework had not covered:
- Changeover/Measurement board sheets carried a ghost 17th
  column (from the standard template) whose date formulas pointed
  at the pre-compaction rows 45..51 - cleared; the real date
  column is P there.
- Diag programming-tests sheet: two date formulas drifted to
  rows 4/3; normalized to their own rows.
Re-scan: 669 date formulas, 0 wrong-row; all 14 practical sheets
sorted بالا/متوسط/پایین with the 'چه چیزی باید ببینید' column.
Both gates green.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -1849,10 +1849,7 @@
         <f>IF(OR(K5="",K5="در انتظار"),"",IF(P5="",TODAY(),P5))</f>
         <v/>
       </c>
-      <c r="Q5" s="103">
-        <f>IF(OR(L45="",L45="در انتظار"),"",IF(Q45="",TODAY(),Q45))</f>
-        <v/>
-      </c>
+      <c r="Q5" s="103" t="n"/>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="99" t="inlineStr">
@@ -1921,10 +1918,7 @@
         <f>IF(OR(K6="",K6="در انتظار"),"",IF(P6="",TODAY(),P6))</f>
         <v/>
       </c>
-      <c r="Q6" s="107">
-        <f>IF(OR(L46="",L46="در انتظار"),"",IF(Q46="",TODAY(),Q46))</f>
-        <v/>
-      </c>
+      <c r="Q6" s="107" t="n"/>
     </row>
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="99" t="inlineStr">
@@ -1993,10 +1987,7 @@
         <f>IF(OR(K7="",K7="در انتظار"),"",IF(P7="",TODAY(),P7))</f>
         <v/>
       </c>
-      <c r="Q7" s="103">
-        <f>IF(OR(L47="",L47="در انتظار"),"",IF(Q47="",TODAY(),Q47))</f>
-        <v/>
-      </c>
+      <c r="Q7" s="103" t="n"/>
     </row>
     <row r="8" ht="54" customHeight="1">
       <c r="A8" s="99" t="inlineStr">
@@ -2065,10 +2056,7 @@
         <f>IF(OR(K8="",K8="در انتظار"),"",IF(P8="",TODAY(),P8))</f>
         <v/>
       </c>
-      <c r="Q8" s="107">
-        <f>IF(OR(L48="",L48="در انتظار"),"",IF(Q48="",TODAY(),Q48))</f>
-        <v/>
-      </c>
+      <c r="Q8" s="107" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="131" t="n"/>

</xml_diff>

<commit_message>
scenario 8: panel reset key (slot 204), working checkboxes, short Persian card
- card 8: short/simple sections, per-parameter explanation lines, reset button
- cb147/cb157 now write to the board (onchange + draw mirror)
- new command slot 204 -> Changeover weak-verdict reset (STM + both ESP panels)
- user panel: third reset button, queue range 200..204 (len 5)
- tests: changeover host 294, scenario cards 409, panel click 156, ESP 126, user 54
- docs/workbooks: Changeover README + CO-032, ESP READMEs, state-machine tabs

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -5102,21 +5102,69 @@
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="82" t="n"/>
-      <c r="B31" s="82" t="n"/>
-      <c r="C31" s="82" t="n"/>
-      <c r="D31" s="82" t="n"/>
-      <c r="E31" s="82" t="n"/>
-      <c r="F31" s="82" t="n"/>
-      <c r="G31" s="82" t="n"/>
-      <c r="H31" s="82" t="n"/>
-      <c r="I31" s="82" t="n"/>
-      <c r="J31" s="82" t="n"/>
-      <c r="K31" s="82" t="n"/>
-      <c r="L31" s="82" t="n"/>
-      <c r="M31" s="82" t="n"/>
-      <c r="N31" s="82" t="n"/>
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="99" t="inlineStr">
+        <is>
+          <t>CO-032</t>
+        </is>
+      </c>
+      <c r="B31" s="143" t="inlineStr">
+        <is>
+          <t>حکم باتری ضعیف / پاک‌کردن دستی از پنل</t>
+        </is>
+      </c>
+      <c r="C31" s="147" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D31" s="143" t="inlineStr">
+        <is>
+          <t>حکم قفل + پنل کالیبراسیون باز</t>
+        </is>
+      </c>
+      <c r="E31" s="145" t="inlineStr">
+        <is>
+          <t>گام ۱: روی برد حکم را قفل کن: بدون برق شهر وصل شود و داخل پنجرهٔ محافظ دوباره قطع شود.
+گام ۲: در کارت ۸ دکمهٔ «پاک‌کردن حکم» را بزن و تأیید کن.
+گام ۳: خط وضعیت باید «در حال ارسال…» و بعد «پاک شد» نشان دهد.
+گام ۴: چراغ قرمز و بوق باید خاموش شوند.
+گام ۵: دوباره همان دکمه را بزن؛ باید بگوید حکمی نیست و خطا ندهد.</t>
+        </is>
+      </c>
+      <c r="F31" s="144" t="inlineStr">
+        <is>
+          <t>حکم=۱ → دکمهٔ پاک‌کردن حکم</t>
+        </is>
+      </c>
+      <c r="G31" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="143" t="inlineStr">
+        <is>
+          <t>حکم همان لحظه پاک می‌شود؛ چهره خاموش و یک بار وصل دوباره آزاد می‌شود. زدن دوبارهٔ دکمه خطا نمی‌دهد. PASS: حکم پاک شد. FAIL: حکم ماند یا دکمه خطا داد.</t>
+        </is>
+      </c>
+      <c r="I31" s="143" t="inlineStr">
+        <is>
+          <t>PASS: حکم پاک. FAIL: حکم ماند.</t>
+        </is>
+      </c>
+      <c r="J31" s="104" t="n"/>
+      <c r="K31" s="143" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="L31" s="115" t="n"/>
+      <c r="M31" s="104" t="n"/>
+      <c r="N31" s="143" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="O31" s="82" t="n"/>
       <c r="P31" s="82" t="n"/>
       <c r="Q31" s="98">

</xml_diff>

<commit_message>
docs: one test-id space across the three Changeover validation sheets (CO-031 was already the panel-display test)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
+++ b/Firmware/Modules/Changeover/Changeover_Board_Validation.xlsx
@@ -1742,7 +1742,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>آستانهٔ استراحت باتری (شناسهٔ ۱۶۵، پیش‌فرض ۲۵٬۰۰۰ mV): زیر آن بدون برق شهر هیچ وصل و هیچ حکمی نیست. سقف تلاش بدون برق شهر یک است. حکم باتری فرسوده فقط بدون برق شهر نمایش داده می‌شود. در حالت قطع بدون برق شهر، هر سه چراغ و بوق خاموش‌اند. قطع سیم باتری بدون برق شهر بی‌صدا است. شناسه‌های تست با شیت «تست‌های آزمایشگاهی» یکسان شد و CO-031/CO-033/CO-034 اضافه شدند.</t>
+          <t>آستانهٔ استراحت باتری (شناسهٔ ۱۶۵، پیش‌فرض ۲۵٬۰۰۰ mV): زیر آن بدون برق شهر هیچ وصل و هیچ حکمی نیست. سقف تلاش بدون برق شهر یک است. حکم باتری فرسوده فقط بدون برق شهر نمایش داده می‌شود. در حالت قطع بدون برق شهر، هر سه چراغ و بوق خاموش‌اند. قطع سیم باتری بدون برق شهر بی‌صدا است. شناسه‌های تست یکسان شد: هر شناسه در «برنامه تست» نسخهٔ عملی و در «تست‌های آزمایشگاهی» نسخهٔ دقیق همان تست است، و CO-020..CO-023 فقط در «تست‌های برنامه‌نویسی» می‌آیند. CO-032/CO-033/CO-034/CO-035 اضافه شدند.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2755,7 +2755,7 @@
     <row r="15" ht="54" customHeight="1">
       <c r="A15" s="99" t="inlineStr">
         <is>
-          <t>CO-031</t>
+          <t>CO-032</t>
         </is>
       </c>
       <c r="B15" s="104" t="inlineStr">
@@ -2765,48 +2765,48 @@
       </c>
       <c r="C15" s="105" t="inlineStr">
         <is>
-          <t>بالا</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="D15" s="104" t="inlineStr">
         <is>
-          <t>دستگاه بدون برق شهر و مسیر باتری بسته</t>
+          <t>حکم قفل + پنل کالیبراسیون باز</t>
         </is>
       </c>
       <c r="E15" s="104" t="inlineStr">
         <is>
-          <t>گام ۱: بگذار باتری زیر ۲۱ ولت برود تا مسیر بسته شود.
-گام ۲: ولتاژ را روی ۲۳٫۰ ولت نگه دار و ۶۰ ثانیه نگاه کن.
-گام ۳: ولتاژ را به ۲۵٫۵ ولت برسان و ۲۰ ثانیه نگاه کن.
-گام ۴: داخل ۶۰ ثانیه بعد از وصل، دوباره زیر ۲۱ ولت بیاور.</t>
+          <t>گام ۱: روی برد حکم را قفل کن.
+گام ۲: در کارت ۸ دکمهٔ پاک‌کردن حکم را بزن.
+گام ۳: خط وضعیت، چراغ قرمز و بوق را نگاه کن.
+گام ۴: همان دکمه را دوباره بزن.</t>
         </is>
       </c>
       <c r="F15" s="104" t="inlineStr">
         <is>
-          <t>استراحت ۲۳ ولت، سپس ۲۵٫۵ ولت، بدون برق شهر</t>
+          <t>حکم = ۱ → دکمهٔ پاک‌کردن حکم (شناسهٔ ۲۰۴)</t>
         </is>
       </c>
       <c r="G15" s="105" t="inlineStr">
         <is>
-          <t>حدود دو دقیقه</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" s="104" t="inlineStr">
         <is>
-          <t>با ۲۳ ولت هیچ وصل و هیچ حکمی نمی‌شود؛ با ۲۵٫۵ ولت یک بار وصل و با قطع دوباره حکم قفل می‌شود</t>
+          <t>حکم همان لحظه پاک می‌شود، چراغ و بوق خاموش می‌شوند و یک تلاش آزاد می‌شود</t>
         </is>
       </c>
       <c r="I15" s="104" t="inlineStr">
         <is>
           <t>باید ببینید:
-در گام ۲ هیچ وصل خودکاری انجام نمی‌شود و حکمی هم زده نمی‌شود (محافظت باتری، مستقل از تیک سناریو).
-در گام ۳ فقط یک بار وصل می‌شود.
-در گام ۴ دوباره وصل نمی‌شود و حکم باتری فرسوده قفل می‌شود.</t>
+خط وضعیت «در حال ارسال…» و بعد «پاک شد» نشان می‌دهد.
+قرمز و بوق خاموش می‌شوند و با استراحت بالای ۲۵ ولت یک بار دیگر وصل می‌شود.
+زدن دوبارهٔ دکمه خطا نمی‌دهد؛ خود ریست پین را دست نمی‌زند.</t>
         </is>
       </c>
       <c r="J15" s="104" t="inlineStr">
         <is>
-          <t>عدم وصل با ۲۳ ولت + یک تلاش با ۲۵٫۵ ولت؛ وصل با ۲۳ ولت = رد</t>
+          <t>حکم پاک شود و دکمهٔ دوم خطا ندهد</t>
         </is>
       </c>
       <c r="K15" s="100" t="n"/>
@@ -2825,14 +2825,14 @@
       <c r="Q15" s="103" t="n"/>
       <c r="R15" s="157" t="inlineStr">
         <is>
-          <t>بدون فرمول: آستانهٔ استراحت شناسهٔ ۱۶۵ هم برای اجازهٔ وصل و هم برای حکم استفاده می‌شود.</t>
+          <t>بدون فرمول: شناسهٔ ۲۰۴ دستور است، نه پارامتر؛ ذخیره نمی‌شود.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="54" customHeight="1">
       <c r="A16" s="99" t="inlineStr">
         <is>
-          <t>CO-032</t>
+          <t>CO-033</t>
         </is>
       </c>
       <c r="B16" s="104" t="inlineStr">
@@ -2842,48 +2842,48 @@
       </c>
       <c r="C16" s="105" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>بالا</t>
         </is>
       </c>
       <c r="D16" s="104" t="inlineStr">
         <is>
-          <t>حکم قفل + پنل کالیبراسیون باز</t>
+          <t>دستگاه بدون برق شهر و مسیر باتری بسته</t>
         </is>
       </c>
       <c r="E16" s="104" t="inlineStr">
         <is>
-          <t>گام ۱: روی برد حکم را قفل کن.
-گام ۲: در کارت ۸ دکمهٔ پاک‌کردن حکم را بزن.
-گام ۳: خط وضعیت، چراغ قرمز و بوق را نگاه کن.
-گام ۴: همان دکمه را دوباره بزن.</t>
+          <t>گام ۱: بگذار باتری زیر ۲۱ ولت برود تا مسیر بسته شود.
+گام ۲: ولتاژ را روی ۲۳٫۰ ولت نگه دار و ۶۰ ثانیه نگاه کن.
+گام ۳: ولتاژ را به ۲۵٫۵ ولت برسان و ۲۰ ثانیه نگاه کن.
+گام ۴: داخل ۶۰ ثانیه بعد از وصل، دوباره زیر ۲۱ ولت بیاور.</t>
         </is>
       </c>
       <c r="F16" s="104" t="inlineStr">
         <is>
-          <t>حکم = ۱ → دکمهٔ پاک‌کردن حکم (شناسهٔ ۲۰۴)</t>
+          <t>استراحت ۲۳ ولت، سپس ۲۵٫۵ ولت، بدون برق شهر</t>
         </is>
       </c>
       <c r="G16" s="105" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>حدود دو دقیقه</t>
         </is>
       </c>
       <c r="H16" s="104" t="inlineStr">
         <is>
-          <t>حکم همان لحظه پاک می‌شود، چراغ و بوق خاموش می‌شوند و یک تلاش آزاد می‌شود</t>
+          <t>با ۲۳ ولت هیچ وصل و هیچ حکمی نمی‌شود؛ با ۲۵٫۵ ولت یک بار وصل و با قطع دوباره حکم قفل می‌شود</t>
         </is>
       </c>
       <c r="I16" s="104" t="inlineStr">
         <is>
           <t>باید ببینید:
-خط وضعیت «در حال ارسال…» و بعد «پاک شد» نشان می‌دهد.
-قرمز و بوق خاموش می‌شوند و با استراحت بالای ۲۵ ولت یک بار دیگر وصل می‌شود.
-زدن دوبارهٔ دکمه خطا نمی‌دهد؛ خود ریست پین را دست نمی‌زند.</t>
+در گام ۲ هیچ وصل خودکاری انجام نمی‌شود و حکمی هم زده نمی‌شود (محافظت باتری، مستقل از تیک سناریو).
+در گام ۳ فقط یک بار وصل می‌شود.
+در گام ۴ دوباره وصل نمی‌شود و حکم باتری فرسوده قفل می‌شود.</t>
         </is>
       </c>
       <c r="J16" s="104" t="inlineStr">
         <is>
-          <t>حکم پاک شود و دکمهٔ دوم خطا ندهد</t>
+          <t>عدم وصل با ۲۳ ولت + یک تلاش با ۲۵٫۵ ولت؛ وصل با ۲۳ ولت = رد</t>
         </is>
       </c>
       <c r="K16" s="100" t="n"/>
@@ -2902,14 +2902,14 @@
       <c r="Q16" s="103" t="n"/>
       <c r="R16" s="157" t="inlineStr">
         <is>
-          <t>بدون فرمول: شناسهٔ ۲۰۴ دستور است، نه پارامتر؛ ذخیره نمی‌شود.</t>
+          <t>بدون فرمول: آستانهٔ استراحت شناسهٔ ۱۶۵ هم برای اجازهٔ وصل و هم برای حکم استفاده می‌شود.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">
       <c r="A17" s="99" t="inlineStr">
         <is>
-          <t>CO-033</t>
+          <t>CO-034</t>
         </is>
       </c>
       <c r="B17" s="104" t="inlineStr">
@@ -2984,7 +2984,7 @@
     <row r="18" ht="54" customHeight="1">
       <c r="A18" s="99" t="inlineStr">
         <is>
-          <t>CO-034</t>
+          <t>CO-035</t>
         </is>
       </c>
       <c r="B18" s="104" t="inlineStr">
@@ -5637,25 +5637,95 @@
     <row r="31" ht="54" customHeight="1">
       <c r="A31" s="99" t="inlineStr">
         <is>
-          <t>CO-031</t>
+          <t>CO-032</t>
         </is>
       </c>
       <c r="B31" s="143" t="inlineStr">
         <is>
+          <t>حکم باتری ضعیف / پاک‌کردن دستی از پنل</t>
+        </is>
+      </c>
+      <c r="C31" s="147" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D31" s="143" t="inlineStr">
+        <is>
+          <t>حکم قفل + پنل کالیبراسیون باز</t>
+        </is>
+      </c>
+      <c r="E31" s="145" t="inlineStr">
+        <is>
+          <t>گام ۱: روی برد حکم را قفل کن: بدون برق شهر وصل شود و داخل پنجرهٔ محافظ دوباره قطع شود.
+گام ۲: در کارت ۸ دکمهٔ «پاک‌کردن حکم» را بزن و تأیید کن.
+گام ۳: خط وضعیت باید «در حال ارسال…» و بعد «پاک شد» نشان دهد.
+گام ۴: چراغ قرمز و بوق باید خاموش شوند.
+گام ۵: دوباره همان دکمه را بزن؛ باید بگوید حکمی نیست و خطا ندهد.</t>
+        </is>
+      </c>
+      <c r="F31" s="144" t="inlineStr">
+        <is>
+          <t>حکم=۱ → دکمهٔ پاک‌کردن حکم</t>
+        </is>
+      </c>
+      <c r="G31" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="143" t="inlineStr">
+        <is>
+          <t>حکم همان لحظه پاک می‌شود؛ چهره خاموش و یک بار وصل دوباره آزاد می‌شود. زدن دوبارهٔ دکمه خطا نمی‌دهد. PASS: حکم پاک شد. FAIL: حکم ماند یا دکمه خطا داد.</t>
+        </is>
+      </c>
+      <c r="I31" s="143" t="inlineStr">
+        <is>
+          <t>PASS: حکم پاک. FAIL: حکم ماند.</t>
+        </is>
+      </c>
+      <c r="J31" s="104" t="n"/>
+      <c r="K31" s="143" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="L31" s="115" t="n"/>
+      <c r="M31" s="104" t="n"/>
+      <c r="N31" s="143" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="O31" s="82" t="n"/>
+      <c r="P31" s="82" t="n"/>
+      <c r="Q31" s="98">
+        <f>IF(OR(L31="",L31="در انتظار"),"",IF(Q31="",TODAY(),Q31))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="99" t="inlineStr">
+        <is>
+          <t>CO-033</t>
+        </is>
+      </c>
+      <c r="B32" s="143" t="inlineStr">
+        <is>
           <t>آستانهٔ استراحت ۲۵٬۰۰۰ mV / بستهٔ دشارژ وصل نمی‌شود</t>
         </is>
       </c>
-      <c r="C31" s="147" t="inlineStr">
+      <c r="C32" s="147" t="inlineStr">
         <is>
           <t>بالا</t>
         </is>
       </c>
-      <c r="D31" s="143" t="inlineStr">
+      <c r="D32" s="143" t="inlineStr">
         <is>
           <t>برد در SAFE، برق شهر قطع، خروجی قطع</t>
         </is>
       </c>
-      <c r="E31" s="145" t="inlineStr">
+      <c r="E32" s="145" t="inlineStr">
         <is>
           <t>گام ۱: از تست CO-008 شروع کن تا خروجی قطع شود.
 گام ۲: ولتاژ را روی 23000 mV نگه دار و ۶۰ ثانیه بمان.
@@ -5664,94 +5734,24 @@
 گام ۵: داخل ۶۰ ثانیه دوباره زیر 21000 mV بیاور؛ باید حکم قفل شود.</t>
         </is>
       </c>
-      <c r="F31" s="144" t="inlineStr">
+      <c r="F32" s="144" t="inlineStr">
         <is>
           <t>input=false، v=23000 سپس 25500 سپس قطع دوباره</t>
         </is>
       </c>
-      <c r="G31" s="144" t="inlineStr">
+      <c r="G32" s="144" t="inlineStr">
         <is>
           <t>۶۰s + ۲۰s + ۶۰s</t>
         </is>
       </c>
-      <c r="H31" s="143" t="inlineStr">
+      <c r="H32" s="143" t="inlineStr">
         <is>
           <t>با استراحت ۲۳ ولت هیچ وصل و هیچ حکمی نمی‌شود؛ با ۲۵٫۵ ولت فقط یک بار وصل می‌شود و قطع دوباره حکم را قفل می‌کند. PASS: عدم وصل با ۲۳ ولت + یک تلاش با ۲۵٫۵ ولت. FAIL: وصل با ۲۳ ولت یا تلاش دوم.</t>
         </is>
       </c>
-      <c r="I31" s="143" t="inlineStr">
+      <c r="I32" s="143" t="inlineStr">
         <is>
           <t>PASS: ۲۳ ولت بدون وصل، ۲۵٫۵ ولت یک تلاش. FAIL: وصل با ۲۳ ولت.</t>
-        </is>
-      </c>
-      <c r="J31" s="104" t="n"/>
-      <c r="K31" s="143" t="inlineStr">
-        <is>
-          <t>در انتظار</t>
-        </is>
-      </c>
-      <c r="L31" s="115" t="n"/>
-      <c r="M31" s="104" t="n"/>
-      <c r="N31" s="143" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="O31" s="82" t="n"/>
-      <c r="P31" s="82" t="n"/>
-      <c r="Q31" s="98">
-        <f>IF(OR(L31="",L31="در انتظار"),"",IF(Q31="",TODAY(),Q31))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="54" customHeight="1">
-      <c r="A32" s="99" t="inlineStr">
-        <is>
-          <t>CO-032</t>
-        </is>
-      </c>
-      <c r="B32" s="143" t="inlineStr">
-        <is>
-          <t>حکم باتری ضعیف / پاک‌کردن دستی از پنل</t>
-        </is>
-      </c>
-      <c r="C32" s="147" t="inlineStr">
-        <is>
-          <t>بالا</t>
-        </is>
-      </c>
-      <c r="D32" s="143" t="inlineStr">
-        <is>
-          <t>حکم قفل + پنل کالیبراسیون باز</t>
-        </is>
-      </c>
-      <c r="E32" s="145" t="inlineStr">
-        <is>
-          <t>گام ۱: روی برد حکم را قفل کن: بدون برق شهر وصل شود و داخل پنجرهٔ محافظ دوباره قطع شود.
-گام ۲: در کارت ۸ دکمهٔ «پاک‌کردن حکم» را بزن و تأیید کن.
-گام ۳: خط وضعیت باید «در حال ارسال…» و بعد «پاک شد» نشان دهد.
-گام ۴: چراغ قرمز و بوق باید خاموش شوند.
-گام ۵: دوباره همان دکمه را بزن؛ باید بگوید حکمی نیست و خطا ندهد.</t>
-        </is>
-      </c>
-      <c r="F32" s="144" t="inlineStr">
-        <is>
-          <t>حکم=۱ → دکمهٔ پاک‌کردن حکم</t>
-        </is>
-      </c>
-      <c r="G32" s="144" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="143" t="inlineStr">
-        <is>
-          <t>حکم همان لحظه پاک می‌شود؛ چهره خاموش و یک بار وصل دوباره آزاد می‌شود. زدن دوبارهٔ دکمه خطا نمی‌دهد. PASS: حکم پاک شد. FAIL: حکم ماند یا دکمه خطا داد.</t>
-        </is>
-      </c>
-      <c r="I32" s="143" t="inlineStr">
-        <is>
-          <t>PASS: حکم پاک. FAIL: حکم ماند.</t>
         </is>
       </c>
       <c r="J32" s="104" t="n"/>
@@ -5777,7 +5777,7 @@
     <row r="33" ht="54" customHeight="1">
       <c r="A33" s="99" t="inlineStr">
         <is>
-          <t>CO-033</t>
+          <t>CO-034</t>
         </is>
       </c>
       <c r="B33" s="143" t="inlineStr">
@@ -5845,7 +5845,7 @@
     <row r="34" ht="54" customHeight="1">
       <c r="A34" s="99" t="inlineStr">
         <is>
-          <t>CO-034</t>
+          <t>CO-035</t>
         </is>
       </c>
       <c r="B34" s="143" t="inlineStr">

</xml_diff>